<commit_message>
Trasnformation and first tests done
</commit_message>
<xml_diff>
--- a/Diplomski plan checklist.xlsx
+++ b/Diplomski plan checklist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Milic\Desktop\cancer-platform\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\cancer-platform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB56BB7-27D7-4BBC-BCD5-96888D087150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C8B08A-7977-4190-810F-239888F95499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4305" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-274286" yWindow="-274286" windowWidth="2366" windowHeight="386" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="160">
   <si>
     <t>Diplomski plan: Checklist (dataset registry + pipeline + baseline)</t>
   </si>
@@ -498,13 +498,16 @@
   </si>
   <si>
     <t>https://github.com/Milki19/cancer-platform.git</t>
+  </si>
+  <si>
+    <t>In Progress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -844,7 +847,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -858,7 +861,7 @@
     <col min="12" max="12" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="27.95" customHeight="1">
+    <row r="1" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -874,7 +877,7 @@
       <c r="K1" s="12"/>
       <c r="L1" s="12"/>
     </row>
-    <row r="3" spans="1:12" ht="60">
+    <row r="3" spans="1:12" ht="58.3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -887,14 +890,14 @@
       </c>
       <c r="D3" s="1">
         <f>COUNTIF($H$7:$H$61,"Done")</f>
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F3" s="2">
         <f>IF(B3=0,0,D3/B3)</f>
-        <v>0.16363636363636364</v>
+        <v>0.30909090909090908</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>4</v>
@@ -908,10 +911,10 @@
       </c>
       <c r="J3" s="1">
         <f>COUNTIF($H$7:$H$61,"In Progress")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="21.95" customHeight="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
@@ -949,7 +952,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A7" s="4">
         <v>1</v>
       </c>
@@ -976,7 +979,7 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
     </row>
-    <row r="8" spans="1:12" ht="30">
+    <row r="8" spans="1:12" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A8" s="4">
         <v>2</v>
       </c>
@@ -1003,7 +1006,7 @@
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
     </row>
-    <row r="9" spans="1:12" ht="30">
+    <row r="9" spans="1:12" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A9" s="4">
         <v>3</v>
       </c>
@@ -1032,7 +1035,7 @@
       </c>
       <c r="L9" s="5"/>
     </row>
-    <row r="10" spans="1:12" ht="30">
+    <row r="10" spans="1:12" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A10" s="4">
         <v>4</v>
       </c>
@@ -1063,7 +1066,7 @@
       </c>
       <c r="L10" s="5"/>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A11" s="4">
         <v>5</v>
       </c>
@@ -1092,7 +1095,7 @@
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A12" s="4">
         <v>6</v>
       </c>
@@ -1121,7 +1124,7 @@
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A13" s="4">
         <v>7</v>
       </c>
@@ -1150,7 +1153,7 @@
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
     </row>
-    <row r="14" spans="1:12" ht="30">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A14" s="4">
         <v>8</v>
       </c>
@@ -1179,7 +1182,7 @@
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A15" s="4">
         <v>9</v>
       </c>
@@ -1206,7 +1209,7 @@
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A16" s="4">
         <v>10</v>
       </c>
@@ -1225,17 +1228,17 @@
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
     </row>
-    <row r="17" spans="1:12" ht="30">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A17" s="4">
         <v>11</v>
       </c>
@@ -1254,17 +1257,17 @@
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I17" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18" s="4">
         <v>12</v>
       </c>
@@ -1293,7 +1296,7 @@
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A19" s="4">
         <v>13</v>
       </c>
@@ -1322,7 +1325,7 @@
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A20" s="4">
         <v>14</v>
       </c>
@@ -1351,7 +1354,7 @@
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A21" s="4">
         <v>15</v>
       </c>
@@ -1368,17 +1371,17 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I21" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" s="4"/>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A22" s="4">
         <v>16</v>
       </c>
@@ -1405,7 +1408,7 @@
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23" s="4">
         <v>17</v>
       </c>
@@ -1422,17 +1425,17 @@
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I23" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" s="4"/>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
     </row>
-    <row r="24" spans="1:12" ht="30">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A24" s="4">
         <v>18</v>
       </c>
@@ -1449,17 +1452,17 @@
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I24" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" s="4"/>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25" s="4">
         <v>19</v>
       </c>
@@ -1488,7 +1491,7 @@
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A26" s="4">
         <v>20</v>
       </c>
@@ -1515,7 +1518,7 @@
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27" s="4">
         <v>21</v>
       </c>
@@ -1544,7 +1547,7 @@
       <c r="K27" s="5"/>
       <c r="L27" s="5"/>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A28" s="4">
         <v>22</v>
       </c>
@@ -1573,7 +1576,7 @@
       <c r="K28" s="5"/>
       <c r="L28" s="5"/>
     </row>
-    <row r="29" spans="1:12" ht="30">
+    <row r="29" spans="1:12" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A29" s="4">
         <v>23</v>
       </c>
@@ -1602,7 +1605,7 @@
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A30" s="4">
         <v>24</v>
       </c>
@@ -1621,17 +1624,17 @@
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
-        <v>21</v>
+        <v>159</v>
       </c>
       <c r="I30" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>IF($H30="Done",1,IF($H30="In Progress",0.5,0))</f>
+        <v>0.5</v>
       </c>
       <c r="J30" s="4"/>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A31" s="4">
         <v>25</v>
       </c>
@@ -1660,7 +1663,7 @@
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A32" s="4">
         <v>26</v>
       </c>
@@ -1679,17 +1682,17 @@
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I32" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" s="4"/>
       <c r="K32" s="5"/>
       <c r="L32" s="5"/>
     </row>
-    <row r="33" spans="1:12">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A33" s="4">
         <v>27</v>
       </c>
@@ -1708,17 +1711,17 @@
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I33" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" s="4"/>
       <c r="K33" s="5"/>
       <c r="L33" s="5"/>
     </row>
-    <row r="34" spans="1:12">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A34" s="4">
         <v>28</v>
       </c>
@@ -1747,7 +1750,7 @@
       <c r="K34" s="5"/>
       <c r="L34" s="5"/>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A35" s="4">
         <v>29</v>
       </c>
@@ -1776,7 +1779,7 @@
       <c r="K35" s="5"/>
       <c r="L35" s="5"/>
     </row>
-    <row r="36" spans="1:12">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A36" s="4">
         <v>30</v>
       </c>
@@ -1803,7 +1806,7 @@
       <c r="K36" s="5"/>
       <c r="L36" s="5"/>
     </row>
-    <row r="37" spans="1:12" ht="30">
+    <row r="37" spans="1:12" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A37" s="4">
         <v>31</v>
       </c>
@@ -1830,7 +1833,7 @@
       <c r="K37" s="5"/>
       <c r="L37" s="5"/>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A38" s="4">
         <v>32</v>
       </c>
@@ -1857,7 +1860,7 @@
       <c r="K38" s="5"/>
       <c r="L38" s="5"/>
     </row>
-    <row r="39" spans="1:12">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A39" s="4">
         <v>33</v>
       </c>
@@ -1884,7 +1887,7 @@
       <c r="K39" s="5"/>
       <c r="L39" s="5"/>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A40" s="4">
         <v>34</v>
       </c>
@@ -1911,7 +1914,7 @@
       <c r="K40" s="5"/>
       <c r="L40" s="5"/>
     </row>
-    <row r="41" spans="1:12">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A41" s="4">
         <v>35</v>
       </c>
@@ -1938,7 +1941,7 @@
       <c r="K41" s="5"/>
       <c r="L41" s="5"/>
     </row>
-    <row r="42" spans="1:12" ht="30">
+    <row r="42" spans="1:12" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A42" s="4">
         <v>36</v>
       </c>
@@ -1967,7 +1970,7 @@
       <c r="K42" s="5"/>
       <c r="L42" s="5"/>
     </row>
-    <row r="43" spans="1:12">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A43" s="4">
         <v>37</v>
       </c>
@@ -1996,7 +1999,7 @@
       <c r="K43" s="5"/>
       <c r="L43" s="5"/>
     </row>
-    <row r="44" spans="1:12">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A44" s="4">
         <v>38</v>
       </c>
@@ -2025,7 +2028,7 @@
       <c r="K44" s="5"/>
       <c r="L44" s="5"/>
     </row>
-    <row r="45" spans="1:12">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A45" s="4">
         <v>39</v>
       </c>
@@ -2052,7 +2055,7 @@
       <c r="K45" s="5"/>
       <c r="L45" s="5"/>
     </row>
-    <row r="46" spans="1:12">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A46" s="4">
         <v>40</v>
       </c>
@@ -2079,7 +2082,7 @@
       <c r="K46" s="5"/>
       <c r="L46" s="5"/>
     </row>
-    <row r="47" spans="1:12">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A47" s="4">
         <v>41</v>
       </c>
@@ -2106,7 +2109,7 @@
       <c r="K47" s="5"/>
       <c r="L47" s="5"/>
     </row>
-    <row r="48" spans="1:12">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A48" s="4">
         <v>42</v>
       </c>
@@ -2123,17 +2126,17 @@
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I48" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48" s="4"/>
       <c r="K48" s="5"/>
       <c r="L48" s="5"/>
     </row>
-    <row r="49" spans="1:12">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A49" s="4">
         <v>43</v>
       </c>
@@ -2162,7 +2165,7 @@
       <c r="K49" s="5"/>
       <c r="L49" s="5"/>
     </row>
-    <row r="50" spans="1:12">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A50" s="4">
         <v>44</v>
       </c>
@@ -2191,7 +2194,7 @@
       <c r="K50" s="5"/>
       <c r="L50" s="5"/>
     </row>
-    <row r="51" spans="1:12">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A51" s="4">
         <v>45</v>
       </c>
@@ -2220,7 +2223,7 @@
       <c r="K51" s="5"/>
       <c r="L51" s="5"/>
     </row>
-    <row r="52" spans="1:12">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A52" s="4">
         <v>46</v>
       </c>
@@ -2249,7 +2252,7 @@
       <c r="K52" s="5"/>
       <c r="L52" s="5"/>
     </row>
-    <row r="53" spans="1:12">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A53" s="4">
         <v>47</v>
       </c>
@@ -2278,7 +2281,7 @@
       <c r="K53" s="5"/>
       <c r="L53" s="5"/>
     </row>
-    <row r="54" spans="1:12">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A54" s="4">
         <v>48</v>
       </c>
@@ -2307,7 +2310,7 @@
       <c r="K54" s="5"/>
       <c r="L54" s="5"/>
     </row>
-    <row r="55" spans="1:12">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A55" s="4">
         <v>49</v>
       </c>
@@ -2336,7 +2339,7 @@
       <c r="K55" s="5"/>
       <c r="L55" s="5"/>
     </row>
-    <row r="56" spans="1:12">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A56" s="4">
         <v>50</v>
       </c>
@@ -2365,7 +2368,7 @@
       <c r="K56" s="5"/>
       <c r="L56" s="5"/>
     </row>
-    <row r="57" spans="1:12">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A57" s="4">
         <v>51</v>
       </c>
@@ -2394,7 +2397,7 @@
       <c r="K57" s="5"/>
       <c r="L57" s="5"/>
     </row>
-    <row r="58" spans="1:12">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A58" s="4">
         <v>52</v>
       </c>
@@ -2423,7 +2426,7 @@
       <c r="K58" s="5"/>
       <c r="L58" s="5"/>
     </row>
-    <row r="59" spans="1:12">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A59" s="4">
         <v>53</v>
       </c>
@@ -2452,7 +2455,7 @@
       <c r="K59" s="5"/>
       <c r="L59" s="5"/>
     </row>
-    <row r="60" spans="1:12">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A60" s="4">
         <v>54</v>
       </c>
@@ -2481,7 +2484,7 @@
       <c r="K60" s="5"/>
       <c r="L60" s="5"/>
     </row>
-    <row r="61" spans="1:12">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A61" s="4">
         <v>55</v>
       </c>
@@ -2541,55 +2544,55 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75">
+    <row r="1" spans="1:1" ht="18.45" x14ac:dyDescent="0.5">
       <c r="A1" s="7" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="18" customHeight="1">
+    <row r="3" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="18" customHeight="1">
+    <row r="4" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="8" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="18" customHeight="1">
+    <row r="5" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="8" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="18" customHeight="1">
+    <row r="6" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="8" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="18" customHeight="1">
+    <row r="7" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="8" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="18" customHeight="1">
+    <row r="8" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="8"/>
     </row>
-    <row r="9" spans="1:1" ht="18" customHeight="1">
+    <row r="9" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="9" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="18" customHeight="1">
+    <row r="10" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="8" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="18" customHeight="1">
+    <row r="11" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="8" t="s">
         <v>155</v>
       </c>

</xml_diff>